<commit_message>
adjusted saving path for the scaler
</commit_message>
<xml_diff>
--- a/Predictions/Extrapolation/Homoserine_Predictions.xlsx
+++ b/Predictions/Extrapolation/Homoserine_Predictions.xlsx
@@ -455,7 +455,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7867080569267273</v>
+        <v>0.7126922011375427</v>
       </c>
     </row>
     <row r="3">
@@ -468,46 +468,46 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7567840218544006</v>
+        <v>0.6889955401420593</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>O=C(NCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCCCCCCCC)=O</t>
+          <t>O=C(NCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCCCCCC)=O</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7460440397262573</v>
+        <v>0.6562804579734802</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>O=C(NCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCCCCCC)=O</t>
+          <t>O=C(NCCCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCC)=O</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7304369807243347</v>
+        <v>0.6551200151443481</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>O=C(NCCCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCC)=O</t>
+          <t>O=C(NCCCCCCCCCCCCCCCC)[C@@H](NC(CCN1CCCC1)=O)CCOC(CCCCCCCCCCC)=O</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6980934739112854</v>
+        <v>0.6409797668457031</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6628809571266174</v>
+        <v>0.6008215546607971</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5003017783164978</v>
+        <v>0.600371778011322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>